<commit_message>
feat: final commit from 1/13/2026
</commit_message>
<xml_diff>
--- a/reference/inflators-1970-2020.xlsx
+++ b/reference/inflators-1970-2020.xlsx
@@ -5,17 +5,19 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ls4540\Documents\dev\households-over-the-years\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ls4540\Documents\dev\households-over-the-years\reference\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C2F8B995-DF19-4863-9085-98EB80713969}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E7A3776-DA3B-48A9-846D-FEBF689F5F87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="14860" activeTab="2" xr2:uid="{1B5009E0-B0EE-4A60-9423-4970FABC966F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="14860" activeTab="4" xr2:uid="{1B5009E0-B0EE-4A60-9423-4970FABC966F}"/>
   </bookViews>
   <sheets>
-    <sheet name="input" sheetId="1" r:id="rId1"/>
-    <sheet name="calculation" sheetId="2" r:id="rId2"/>
-    <sheet name="output" sheetId="3" r:id="rId3"/>
+    <sheet name="inflation-input" sheetId="1" r:id="rId1"/>
+    <sheet name="inflation-calc" sheetId="2" r:id="rId2"/>
+    <sheet name="inflation-output" sheetId="3" r:id="rId3"/>
+    <sheet name="topcode-input" sheetId="5" r:id="rId4"/>
+    <sheet name="topcode-calc" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="63">
   <si>
     <t>Data Year</t>
   </si>
@@ -163,17 +165,80 @@
     <t>https://usa.ipums.org/usa/cpi99.shtml</t>
   </si>
   <si>
-    <t>source_year</t>
-  </si>
-  <si>
     <t>inflator_2020</t>
+  </si>
+  <si>
+    <t>Census</t>
+  </si>
+  <si>
+    <t>Bottom Code</t>
+  </si>
+  <si>
+    <t>Top Code</t>
+  </si>
+  <si>
+    <t>Net loss</t>
+  </si>
+  <si>
+    <t> $400,000*</t>
+  </si>
+  <si>
+    <t>ACS</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>PRCS</t>
+  </si>
+  <si>
+    <t>source:</t>
+  </si>
+  <si>
+    <t>https://usa.ipums.org/usa-action/variables/INCTOT#codes_section</t>
+  </si>
+  <si>
+    <t>year</t>
+  </si>
+  <si>
+    <t>I use the census version rather than the ACS version for 2000</t>
+  </si>
+  <si>
+    <t>to harmonize encoding across years, we pull the largest bottom code and the smallest top code and apply it to all other data.</t>
+  </si>
+  <si>
+    <t>unified bottom code ($2020)</t>
+  </si>
+  <si>
+    <t>bottom code ($contemp)</t>
+  </si>
+  <si>
+    <t>top code ($contemp)</t>
+  </si>
+  <si>
+    <t>bottom code ($2020)</t>
+  </si>
+  <si>
+    <t>top code ($2020)</t>
+  </si>
+  <si>
+    <t>unified top code ($2020)</t>
+  </si>
+  <si>
+    <t>We round the bottom code to -$16,000 and the top code to $250,000</t>
+  </si>
+  <si>
+    <t>YEAR</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <numFmts count="1">
+    <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
+  </numFmts>
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -192,8 +257,21 @@
       <color rgb="FF00263A"/>
       <name val="Cabrito Sans Subset"/>
     </font>
+    <font>
+      <sz val="9.35"/>
+      <color rgb="FF00263A"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF00263A"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -212,8 +290,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -236,17 +320,41 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="6" fontId="3" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1260,14 +1368,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{568AEB72-8931-4B22-9FD3-B9B5F0CBA475}">
-  <dimension ref="B2:D31"/>
+  <dimension ref="B2:E30"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="3" max="3" width="13" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4">
+    <row r="2" spans="2:5">
       <c r="B2" t="s">
         <v>38</v>
       </c>
@@ -1278,380 +1386,370 @@
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="2:4">
+    <row r="3" spans="2:5">
       <c r="B3">
         <v>1970</v>
       </c>
       <c r="C3">
-        <f>input!E6</f>
+        <f>'inflation-input'!E6</f>
         <v>4.54</v>
       </c>
       <c r="D3">
-        <f>(1/input!$E$30)*calculation!C3</f>
+        <f>(1/'inflation-input'!$E$30)*'inflation-calc'!C3</f>
         <v>7.0496894409937889</v>
       </c>
     </row>
-    <row r="4" spans="2:4">
+    <row r="4" spans="2:5">
       <c r="B4">
         <v>1980</v>
       </c>
       <c r="C4">
-        <f>input!E7</f>
+        <f>'inflation-input'!E7</f>
         <v>2.2949999999999999</v>
       </c>
       <c r="D4">
-        <f>(1/input!$E$30)*calculation!C4</f>
+        <f>(1/'inflation-input'!$E$30)*'inflation-calc'!C4</f>
         <v>3.5636645962732918</v>
       </c>
     </row>
-    <row r="5" spans="2:4">
+    <row r="5" spans="2:5">
       <c r="B5">
         <v>1990</v>
       </c>
       <c r="C5">
-        <f>input!E8</f>
+        <f>'inflation-input'!E8</f>
         <v>1.3440000000000001</v>
       </c>
       <c r="D5">
-        <f>(1/input!$E$30)*calculation!C5</f>
+        <f>(1/'inflation-input'!$E$30)*'inflation-calc'!C5</f>
         <v>2.0869565217391308</v>
       </c>
     </row>
-    <row r="6" spans="2:4">
+    <row r="6" spans="2:5">
       <c r="B6">
         <v>2000</v>
       </c>
       <c r="C6">
-        <f>input!E9</f>
+        <f>'inflation-input'!E9</f>
         <v>1</v>
       </c>
       <c r="D6">
-        <f>(1/input!$E$30)*calculation!C6</f>
+        <f>(1/'inflation-input'!$E$30)*'inflation-calc'!C6</f>
         <v>1.5527950310559007</v>
       </c>
-    </row>
-    <row r="7" spans="2:4">
+      <c r="E6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5">
       <c r="B7">
-        <v>2000</v>
+        <v>2001</v>
       </c>
       <c r="C7">
-        <f>input!E10</f>
-        <v>0.96699999999999997</v>
+        <f>'inflation-input'!E11</f>
+        <v>0.94099999999999995</v>
       </c>
       <c r="D7">
-        <f>(1/input!$E$30)*calculation!C7</f>
-        <v>1.5015527950310559</v>
-      </c>
-    </row>
-    <row r="8" spans="2:4">
+        <f>(1/'inflation-input'!$E$30)*'inflation-calc'!C7</f>
+        <v>1.4611801242236024</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5">
       <c r="B8">
-        <v>2001</v>
+        <v>2002</v>
       </c>
       <c r="C8">
-        <f>input!E11</f>
-        <v>0.94099999999999995</v>
+        <f>'inflation-input'!E12</f>
+        <v>0.92600000000000005</v>
       </c>
       <c r="D8">
-        <f>(1/input!$E$30)*calculation!C8</f>
-        <v>1.4611801242236024</v>
-      </c>
-    </row>
-    <row r="9" spans="2:4">
+        <f>(1/'inflation-input'!$E$30)*'inflation-calc'!C8</f>
+        <v>1.4378881987577641</v>
+      </c>
+    </row>
+    <row r="9" spans="2:5">
       <c r="B9">
-        <v>2002</v>
+        <v>2003</v>
       </c>
       <c r="C9">
-        <f>input!E12</f>
-        <v>0.92600000000000005</v>
+        <f>'inflation-input'!E13</f>
+        <v>0.90500000000000003</v>
       </c>
       <c r="D9">
-        <f>(1/input!$E$30)*calculation!C9</f>
-        <v>1.4378881987577641</v>
-      </c>
-    </row>
-    <row r="10" spans="2:4">
+        <f>(1/'inflation-input'!$E$30)*'inflation-calc'!C9</f>
+        <v>1.4052795031055902</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5">
       <c r="B10">
-        <v>2003</v>
+        <v>2004</v>
       </c>
       <c r="C10">
-        <f>input!E13</f>
-        <v>0.90500000000000003</v>
+        <f>'inflation-input'!E14</f>
+        <v>0.88200000000000001</v>
       </c>
       <c r="D10">
-        <f>(1/input!$E$30)*calculation!C10</f>
-        <v>1.4052795031055902</v>
-      </c>
-    </row>
-    <row r="11" spans="2:4">
+        <f>(1/'inflation-input'!$E$30)*'inflation-calc'!C10</f>
+        <v>1.3695652173913044</v>
+      </c>
+    </row>
+    <row r="11" spans="2:5">
       <c r="B11">
-        <v>2004</v>
+        <v>2005</v>
       </c>
       <c r="C11">
-        <f>input!E14</f>
-        <v>0.88200000000000001</v>
+        <f>'inflation-input'!E15</f>
+        <v>0.85299999999999998</v>
       </c>
       <c r="D11">
-        <f>(1/input!$E$30)*calculation!C11</f>
-        <v>1.3695652173913044</v>
-      </c>
-    </row>
-    <row r="12" spans="2:4">
+        <f>(1/'inflation-input'!$E$30)*'inflation-calc'!C11</f>
+        <v>1.3245341614906831</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5">
       <c r="B12">
-        <v>2005</v>
+        <v>2006</v>
       </c>
       <c r="C12">
-        <f>input!E15</f>
-        <v>0.85299999999999998</v>
+        <f>'inflation-input'!E16</f>
+        <v>0.82599999999999996</v>
       </c>
       <c r="D12">
-        <f>(1/input!$E$30)*calculation!C12</f>
-        <v>1.3245341614906831</v>
-      </c>
-    </row>
-    <row r="13" spans="2:4">
+        <f>(1/'inflation-input'!$E$30)*'inflation-calc'!C12</f>
+        <v>1.2826086956521738</v>
+      </c>
+    </row>
+    <row r="13" spans="2:5">
       <c r="B13">
-        <v>2006</v>
+        <v>2007</v>
       </c>
       <c r="C13">
-        <f>input!E16</f>
-        <v>0.82599999999999996</v>
+        <f>'inflation-input'!E17</f>
+        <v>0.80400000000000005</v>
       </c>
       <c r="D13">
-        <f>(1/input!$E$30)*calculation!C13</f>
-        <v>1.2826086956521738</v>
-      </c>
-    </row>
-    <row r="14" spans="2:4">
+        <f>(1/'inflation-input'!$E$30)*'inflation-calc'!C13</f>
+        <v>1.2484472049689441</v>
+      </c>
+    </row>
+    <row r="14" spans="2:5">
       <c r="B14">
-        <v>2007</v>
+        <v>2008</v>
       </c>
       <c r="C14">
-        <f>input!E17</f>
-        <v>0.80400000000000005</v>
+        <f>'inflation-input'!E18</f>
+        <v>0.77400000000000002</v>
       </c>
       <c r="D14">
-        <f>(1/input!$E$30)*calculation!C14</f>
-        <v>1.2484472049689441</v>
-      </c>
-    </row>
-    <row r="15" spans="2:4">
+        <f>(1/'inflation-input'!$E$30)*'inflation-calc'!C14</f>
+        <v>1.2018633540372672</v>
+      </c>
+    </row>
+    <row r="15" spans="2:5">
       <c r="B15">
-        <v>2008</v>
+        <v>2009</v>
       </c>
       <c r="C15">
-        <f>input!E18</f>
-        <v>0.77400000000000002</v>
+        <f>'inflation-input'!E19</f>
+        <v>0.77700000000000002</v>
       </c>
       <c r="D15">
-        <f>(1/input!$E$30)*calculation!C15</f>
-        <v>1.2018633540372672</v>
-      </c>
-    </row>
-    <row r="16" spans="2:4">
+        <f>(1/'inflation-input'!$E$30)*'inflation-calc'!C15</f>
+        <v>1.2065217391304348</v>
+      </c>
+    </row>
+    <row r="16" spans="2:5">
       <c r="B16">
-        <v>2009</v>
+        <v>2010</v>
       </c>
       <c r="C16">
-        <f>input!E19</f>
-        <v>0.77700000000000002</v>
+        <f>'inflation-input'!E20</f>
+        <v>0.76400000000000001</v>
       </c>
       <c r="D16">
-        <f>(1/input!$E$30)*calculation!C16</f>
-        <v>1.2065217391304348</v>
+        <f>(1/'inflation-input'!$E$30)*'inflation-calc'!C16</f>
+        <v>1.1863354037267082</v>
       </c>
     </row>
     <row r="17" spans="2:4">
       <c r="B17">
-        <v>2010</v>
+        <v>2011</v>
       </c>
       <c r="C17">
-        <f>input!E20</f>
-        <v>0.76400000000000001</v>
+        <f>'inflation-input'!E21</f>
+        <v>0.74099999999999999</v>
       </c>
       <c r="D17">
-        <f>(1/input!$E$30)*calculation!C17</f>
-        <v>1.1863354037267082</v>
+        <f>(1/'inflation-input'!$E$30)*'inflation-calc'!C17</f>
+        <v>1.1506211180124224</v>
       </c>
     </row>
     <row r="18" spans="2:4">
       <c r="B18">
-        <v>2011</v>
+        <v>2012</v>
       </c>
       <c r="C18">
-        <f>input!E21</f>
-        <v>0.74099999999999999</v>
+        <f>'inflation-input'!E22</f>
+        <v>0.72599999999999998</v>
       </c>
       <c r="D18">
-        <f>(1/input!$E$30)*calculation!C18</f>
-        <v>1.1506211180124224</v>
+        <f>(1/'inflation-input'!$E$30)*'inflation-calc'!C18</f>
+        <v>1.1273291925465838</v>
       </c>
     </row>
     <row r="19" spans="2:4">
       <c r="B19">
-        <v>2012</v>
+        <v>2013</v>
       </c>
       <c r="C19">
-        <f>input!E22</f>
-        <v>0.72599999999999998</v>
+        <f>'inflation-input'!E23</f>
+        <v>0.71499999999999997</v>
       </c>
       <c r="D19">
-        <f>(1/input!$E$30)*calculation!C19</f>
-        <v>1.1273291925465838</v>
+        <f>(1/'inflation-input'!$E$30)*'inflation-calc'!C19</f>
+        <v>1.110248447204969</v>
       </c>
     </row>
     <row r="20" spans="2:4">
       <c r="B20">
-        <v>2013</v>
+        <v>2014</v>
       </c>
       <c r="C20">
-        <f>input!E23</f>
-        <v>0.71499999999999997</v>
+        <f>'inflation-input'!E24</f>
+        <v>0.70399999999999996</v>
       </c>
       <c r="D20">
-        <f>(1/input!$E$30)*calculation!C20</f>
-        <v>1.110248447204969</v>
+        <f>(1/'inflation-input'!$E$30)*'inflation-calc'!C20</f>
+        <v>1.0931677018633541</v>
       </c>
     </row>
     <row r="21" spans="2:4">
       <c r="B21">
-        <v>2014</v>
+        <v>2015</v>
       </c>
       <c r="C21">
-        <f>input!E24</f>
-        <v>0.70399999999999996</v>
+        <f>'inflation-input'!E25</f>
+        <v>0.70299999999999996</v>
       </c>
       <c r="D21">
-        <f>(1/input!$E$30)*calculation!C21</f>
-        <v>1.0931677018633541</v>
+        <f>(1/'inflation-input'!$E$30)*'inflation-calc'!C21</f>
+        <v>1.091614906832298</v>
       </c>
     </row>
     <row r="22" spans="2:4">
       <c r="B22">
-        <v>2015</v>
+        <v>2016</v>
       </c>
       <c r="C22">
-        <f>input!E25</f>
-        <v>0.70299999999999996</v>
+        <f>'inflation-input'!E26</f>
+        <v>0.69399999999999995</v>
       </c>
       <c r="D22">
-        <f>(1/input!$E$30)*calculation!C22</f>
-        <v>1.091614906832298</v>
+        <f>(1/'inflation-input'!$E$30)*'inflation-calc'!C22</f>
+        <v>1.0776397515527949</v>
       </c>
     </row>
     <row r="23" spans="2:4">
       <c r="B23">
-        <v>2016</v>
+        <v>2017</v>
       </c>
       <c r="C23">
-        <f>input!E26</f>
-        <v>0.69399999999999995</v>
+        <f>'inflation-input'!E27</f>
+        <v>0.67900000000000005</v>
       </c>
       <c r="D23">
-        <f>(1/input!$E$30)*calculation!C23</f>
-        <v>1.0776397515527949</v>
+        <f>(1/'inflation-input'!$E$30)*'inflation-calc'!C23</f>
+        <v>1.0543478260869565</v>
       </c>
     </row>
     <row r="24" spans="2:4">
       <c r="B24">
-        <v>2017</v>
+        <v>2018</v>
       </c>
       <c r="C24">
-        <f>input!E27</f>
-        <v>0.67900000000000005</v>
+        <f>'inflation-input'!E28</f>
+        <v>0.66300000000000003</v>
       </c>
       <c r="D24">
-        <f>(1/input!$E$30)*calculation!C24</f>
-        <v>1.0543478260869565</v>
+        <f>(1/'inflation-input'!$E$30)*'inflation-calc'!C24</f>
+        <v>1.0295031055900621</v>
       </c>
     </row>
     <row r="25" spans="2:4">
       <c r="B25">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="C25">
-        <f>input!E28</f>
-        <v>0.66300000000000003</v>
+        <f>'inflation-input'!E29</f>
+        <v>0.65200000000000002</v>
       </c>
       <c r="D25">
-        <f>(1/input!$E$30)*calculation!C25</f>
-        <v>1.0295031055900621</v>
+        <f>(1/'inflation-input'!$E$30)*'inflation-calc'!C25</f>
+        <v>1.0124223602484472</v>
       </c>
     </row>
     <row r="26" spans="2:4">
       <c r="B26">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="C26">
-        <f>input!E29</f>
-        <v>0.65200000000000002</v>
+        <f>'inflation-input'!E30</f>
+        <v>0.64400000000000002</v>
       </c>
       <c r="D26">
-        <f>(1/input!$E$30)*calculation!C26</f>
-        <v>1.0124223602484472</v>
+        <f>(1/'inflation-input'!$E$30)*'inflation-calc'!C26</f>
+        <v>1</v>
       </c>
     </row>
     <row r="27" spans="2:4">
       <c r="B27">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="C27">
-        <f>input!E30</f>
-        <v>0.64400000000000002</v>
+        <f>'inflation-input'!E31</f>
+        <v>0.61499999999999999</v>
       </c>
       <c r="D27">
-        <f>(1/input!$E$30)*calculation!C27</f>
-        <v>1</v>
+        <f>(1/'inflation-input'!$E$30)*'inflation-calc'!C27</f>
+        <v>0.95496894409937894</v>
       </c>
     </row>
     <row r="28" spans="2:4">
       <c r="B28">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="C28">
-        <f>input!E31</f>
-        <v>0.61499999999999999</v>
+        <f>'inflation-input'!E32</f>
+        <v>0.56899999999999995</v>
       </c>
       <c r="D28">
-        <f>(1/input!$E$30)*calculation!C28</f>
-        <v>0.95496894409937894</v>
+        <f>(1/'inflation-input'!$E$30)*'inflation-calc'!C28</f>
+        <v>0.88354037267080743</v>
       </c>
     </row>
     <row r="29" spans="2:4">
       <c r="B29">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="C29">
-        <f>input!E32</f>
-        <v>0.56899999999999995</v>
+        <f>'inflation-input'!E33</f>
+        <v>0.54700000000000004</v>
       </c>
       <c r="D29">
-        <f>(1/input!$E$30)*calculation!C29</f>
-        <v>0.88354037267080743</v>
+        <f>(1/'inflation-input'!$E$30)*'inflation-calc'!C29</f>
+        <v>0.84937888198757772</v>
       </c>
     </row>
     <row r="30" spans="2:4">
       <c r="B30">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="C30">
-        <f>input!E33</f>
-        <v>0.54700000000000004</v>
+        <f>'inflation-input'!E34</f>
+        <v>0.53100000000000003</v>
       </c>
       <c r="D30">
-        <f>(1/input!$E$30)*calculation!C30</f>
-        <v>0.84937888198757772</v>
-      </c>
-    </row>
-    <row r="31" spans="2:4">
-      <c r="B31">
-        <v>2024</v>
-      </c>
-      <c r="C31">
-        <f>input!E34</f>
-        <v>0.53100000000000003</v>
-      </c>
-      <c r="D31">
-        <f>(1/input!$E$30)*calculation!C31</f>
+        <f>(1/'inflation-input'!$E$30)*'inflation-calc'!C30</f>
         <v>0.82453416149068326</v>
       </c>
     </row>
@@ -1662,15 +1760,15 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4A83E91-0B63-45FD-9908-2B23A3F32FFB}">
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B1" t="s">
         <v>41</v>
-      </c>
-      <c r="B1" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -1707,205 +1805,1096 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6">
-        <v>2000</v>
+        <v>2001</v>
       </c>
       <c r="B6">
-        <v>1.5015527950310559</v>
+        <v>1.4611801242236024</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7">
-        <v>2001</v>
+        <v>2002</v>
       </c>
       <c r="B7">
-        <v>1.4611801242236024</v>
+        <v>1.4378881987577641</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8">
-        <v>2002</v>
+        <v>2003</v>
       </c>
       <c r="B8">
-        <v>1.4378881987577641</v>
+        <v>1.4052795031055902</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9">
-        <v>2003</v>
+        <v>2004</v>
       </c>
       <c r="B9">
-        <v>1.4052795031055902</v>
+        <v>1.3695652173913044</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10">
-        <v>2004</v>
+        <v>2005</v>
       </c>
       <c r="B10">
-        <v>1.3695652173913044</v>
+        <v>1.3245341614906831</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11">
-        <v>2005</v>
+        <v>2006</v>
       </c>
       <c r="B11">
-        <v>1.3245341614906831</v>
+        <v>1.2826086956521738</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12">
-        <v>2006</v>
+        <v>2007</v>
       </c>
       <c r="B12">
-        <v>1.2826086956521738</v>
+        <v>1.2484472049689441</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13">
-        <v>2007</v>
+        <v>2008</v>
       </c>
       <c r="B13">
-        <v>1.2484472049689441</v>
+        <v>1.2018633540372672</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14">
-        <v>2008</v>
+        <v>2009</v>
       </c>
       <c r="B14">
-        <v>1.2018633540372672</v>
+        <v>1.2065217391304348</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15">
-        <v>2009</v>
+        <v>2010</v>
       </c>
       <c r="B15">
-        <v>1.2065217391304348</v>
+        <v>1.1863354037267082</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16">
-        <v>2010</v>
+        <v>2011</v>
       </c>
       <c r="B16">
-        <v>1.1863354037267082</v>
+        <v>1.1506211180124224</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17">
-        <v>2011</v>
+        <v>2012</v>
       </c>
       <c r="B17">
-        <v>1.1506211180124224</v>
+        <v>1.1273291925465838</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18">
-        <v>2012</v>
+        <v>2013</v>
       </c>
       <c r="B18">
-        <v>1.1273291925465838</v>
+        <v>1.110248447204969</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19">
-        <v>2013</v>
+        <v>2014</v>
       </c>
       <c r="B19">
-        <v>1.110248447204969</v>
+        <v>1.0931677018633541</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20">
-        <v>2014</v>
+        <v>2015</v>
       </c>
       <c r="B20">
-        <v>1.0931677018633541</v>
+        <v>1.091614906832298</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21">
-        <v>2015</v>
+        <v>2016</v>
       </c>
       <c r="B21">
-        <v>1.091614906832298</v>
+        <v>1.0776397515527949</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22">
-        <v>2016</v>
+        <v>2017</v>
       </c>
       <c r="B22">
-        <v>1.0776397515527949</v>
+        <v>1.0543478260869565</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23">
-        <v>2017</v>
+        <v>2018</v>
       </c>
       <c r="B23">
-        <v>1.0543478260869565</v>
+        <v>1.0295031055900621</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="B24">
-        <v>1.0295031055900621</v>
+        <v>1.0124223602484472</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="B25">
-        <v>1.0124223602484472</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="B26">
-        <v>1</v>
+        <v>0.95496894409937894</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="B27">
-        <v>0.95496894409937894</v>
+        <v>0.88354037267080743</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="B28">
-        <v>0.88354037267080743</v>
+        <v>0.84937888198757772</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="B29">
-        <v>0.84937888198757772</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2">
-      <c r="A30">
-        <v>2024</v>
-      </c>
-      <c r="B30">
         <v>0.82453416149068326</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E297D31-2EE2-41FA-8D4B-8DE05C7AC45D}">
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="13.28515625" customWidth="1"/>
+    <col min="3" max="3" width="16.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="3">
+        <v>1950</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C3" s="5">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="3">
+        <v>1960</v>
+      </c>
+      <c r="B4" s="5">
+        <v>-9900</v>
+      </c>
+      <c r="C4" s="5">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" s="3">
+        <v>1970</v>
+      </c>
+      <c r="B5" s="5">
+        <v>-9900</v>
+      </c>
+      <c r="C5" s="5">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" s="3">
+        <v>1980</v>
+      </c>
+      <c r="B6" s="5">
+        <v>-9990</v>
+      </c>
+      <c r="C6" s="5">
+        <v>75000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" s="3">
+        <v>1990</v>
+      </c>
+      <c r="B7" s="5">
+        <v>-19998</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" s="3">
+        <v>2000</v>
+      </c>
+      <c r="B8" s="5">
+        <v>-20000</v>
+      </c>
+      <c r="C8" s="5">
+        <v>999998</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="5">
+        <v>-19998</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B10" s="5">
+        <v>-19998</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01E406EE-FAF9-45CE-AC8D-F9C85E61A894}">
+  <dimension ref="A1:H32"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="26.28515625" customWidth="1"/>
+    <col min="3" max="4" width="21" customWidth="1"/>
+    <col min="5" max="5" width="20.5703125" customWidth="1"/>
+    <col min="6" max="6" width="16.140625" customWidth="1"/>
+    <col min="7" max="7" width="25.5703125" customWidth="1"/>
+    <col min="8" max="8" width="23.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8">
+      <c r="B1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="B2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" t="s">
+        <v>52</v>
+      </c>
+      <c r="B4" t="s">
+        <v>56</v>
+      </c>
+      <c r="C4" t="s">
+        <v>57</v>
+      </c>
+      <c r="D4" t="s">
+        <v>41</v>
+      </c>
+      <c r="E4" t="s">
+        <v>58</v>
+      </c>
+      <c r="F4" t="s">
+        <v>59</v>
+      </c>
+      <c r="G4" t="s">
+        <v>55</v>
+      </c>
+      <c r="H4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5">
+        <v>1970</v>
+      </c>
+      <c r="B5">
+        <v>-9900</v>
+      </c>
+      <c r="C5">
+        <v>50000</v>
+      </c>
+      <c r="D5">
+        <f>'inflation-output'!B2</f>
+        <v>7.0496894409937889</v>
+      </c>
+      <c r="E5">
+        <f>B5*$D5</f>
+        <v>-69791.925465838503</v>
+      </c>
+      <c r="F5">
+        <f>C5*$D5</f>
+        <v>352484.47204968944</v>
+      </c>
+      <c r="G5">
+        <f t="shared" ref="G5:G32" si="0">MAX(E$5:E$32)</f>
+        <v>-16489.034161490683</v>
+      </c>
+      <c r="H5">
+        <f>MIN(F$5:F$32)</f>
+        <v>267274.84472049691</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6">
+        <v>1980</v>
+      </c>
+      <c r="B6">
+        <v>-9990</v>
+      </c>
+      <c r="C6">
+        <v>75000</v>
+      </c>
+      <c r="D6">
+        <f>'inflation-output'!B3</f>
+        <v>3.5636645962732918</v>
+      </c>
+      <c r="E6">
+        <f t="shared" ref="E6:E32" si="1">B6*$D6</f>
+        <v>-35601.009316770185</v>
+      </c>
+      <c r="F6">
+        <f t="shared" ref="F6:F8" si="2">C6*$D6</f>
+        <v>267274.84472049691</v>
+      </c>
+      <c r="G6">
+        <f t="shared" si="0"/>
+        <v>-16489.034161490683</v>
+      </c>
+      <c r="H6">
+        <f t="shared" ref="H6:H32" si="3">MIN(F$5:F$32)</f>
+        <v>267274.84472049691</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7">
+        <v>1990</v>
+      </c>
+      <c r="B7">
+        <v>-19998</v>
+      </c>
+      <c r="C7">
+        <v>400000</v>
+      </c>
+      <c r="D7">
+        <f>'inflation-output'!B4</f>
+        <v>2.0869565217391308</v>
+      </c>
+      <c r="E7">
+        <f t="shared" si="1"/>
+        <v>-41734.956521739135</v>
+      </c>
+      <c r="F7">
+        <f t="shared" si="2"/>
+        <v>834782.60869565234</v>
+      </c>
+      <c r="G7">
+        <f t="shared" si="0"/>
+        <v>-16489.034161490683</v>
+      </c>
+      <c r="H7">
+        <f t="shared" si="3"/>
+        <v>267274.84472049691</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8">
+        <v>2000</v>
+      </c>
+      <c r="B8">
+        <v>-20000</v>
+      </c>
+      <c r="C8">
+        <v>999998</v>
+      </c>
+      <c r="D8">
+        <f>'inflation-output'!B5</f>
+        <v>1.5527950310559007</v>
+      </c>
+      <c r="E8">
+        <f t="shared" si="1"/>
+        <v>-31055.900621118013</v>
+      </c>
+      <c r="F8">
+        <f t="shared" si="2"/>
+        <v>1552791.9254658385</v>
+      </c>
+      <c r="G8">
+        <f t="shared" si="0"/>
+        <v>-16489.034161490683</v>
+      </c>
+      <c r="H8">
+        <f t="shared" si="3"/>
+        <v>267274.84472049691</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9">
+        <v>2001</v>
+      </c>
+      <c r="B9">
+        <v>-19998</v>
+      </c>
+      <c r="D9">
+        <f>'inflation-output'!B6</f>
+        <v>1.4611801242236024</v>
+      </c>
+      <c r="E9">
+        <f t="shared" si="1"/>
+        <v>-29220.680124223603</v>
+      </c>
+      <c r="G9">
+        <f t="shared" si="0"/>
+        <v>-16489.034161490683</v>
+      </c>
+      <c r="H9">
+        <f t="shared" si="3"/>
+        <v>267274.84472049691</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10">
+        <v>2002</v>
+      </c>
+      <c r="B10">
+        <v>-19998</v>
+      </c>
+      <c r="D10">
+        <f>'inflation-output'!B7</f>
+        <v>1.4378881987577641</v>
+      </c>
+      <c r="E10">
+        <f t="shared" si="1"/>
+        <v>-28754.888198757766</v>
+      </c>
+      <c r="G10">
+        <f t="shared" si="0"/>
+        <v>-16489.034161490683</v>
+      </c>
+      <c r="H10">
+        <f t="shared" si="3"/>
+        <v>267274.84472049691</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11">
+        <v>2003</v>
+      </c>
+      <c r="B11">
+        <v>-19998</v>
+      </c>
+      <c r="D11">
+        <f>'inflation-output'!B8</f>
+        <v>1.4052795031055902</v>
+      </c>
+      <c r="E11">
+        <f t="shared" si="1"/>
+        <v>-28102.779503105594</v>
+      </c>
+      <c r="G11">
+        <f t="shared" si="0"/>
+        <v>-16489.034161490683</v>
+      </c>
+      <c r="H11">
+        <f t="shared" si="3"/>
+        <v>267274.84472049691</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12">
+        <v>2004</v>
+      </c>
+      <c r="B12">
+        <v>-19998</v>
+      </c>
+      <c r="D12">
+        <f>'inflation-output'!B9</f>
+        <v>1.3695652173913044</v>
+      </c>
+      <c r="E12">
+        <f t="shared" si="1"/>
+        <v>-27388.565217391308</v>
+      </c>
+      <c r="G12">
+        <f t="shared" si="0"/>
+        <v>-16489.034161490683</v>
+      </c>
+      <c r="H12">
+        <f t="shared" si="3"/>
+        <v>267274.84472049691</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13">
+        <v>2005</v>
+      </c>
+      <c r="B13">
+        <v>-19998</v>
+      </c>
+      <c r="D13">
+        <f>'inflation-output'!B10</f>
+        <v>1.3245341614906831</v>
+      </c>
+      <c r="E13">
+        <f t="shared" si="1"/>
+        <v>-26488.034161490683</v>
+      </c>
+      <c r="G13">
+        <f t="shared" si="0"/>
+        <v>-16489.034161490683</v>
+      </c>
+      <c r="H13">
+        <f t="shared" si="3"/>
+        <v>267274.84472049691</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14">
+        <v>2006</v>
+      </c>
+      <c r="B14">
+        <v>-19998</v>
+      </c>
+      <c r="D14">
+        <f>'inflation-output'!B11</f>
+        <v>1.2826086956521738</v>
+      </c>
+      <c r="E14">
+        <f t="shared" si="1"/>
+        <v>-25649.608695652172</v>
+      </c>
+      <c r="G14">
+        <f t="shared" si="0"/>
+        <v>-16489.034161490683</v>
+      </c>
+      <c r="H14">
+        <f t="shared" si="3"/>
+        <v>267274.84472049691</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15">
+        <v>2007</v>
+      </c>
+      <c r="B15">
+        <v>-19998</v>
+      </c>
+      <c r="D15">
+        <f>'inflation-output'!B12</f>
+        <v>1.2484472049689441</v>
+      </c>
+      <c r="E15">
+        <f t="shared" si="1"/>
+        <v>-24966.447204968943</v>
+      </c>
+      <c r="G15">
+        <f t="shared" si="0"/>
+        <v>-16489.034161490683</v>
+      </c>
+      <c r="H15">
+        <f t="shared" si="3"/>
+        <v>267274.84472049691</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16">
+        <v>2008</v>
+      </c>
+      <c r="B16">
+        <v>-19998</v>
+      </c>
+      <c r="D16">
+        <f>'inflation-output'!B13</f>
+        <v>1.2018633540372672</v>
+      </c>
+      <c r="E16">
+        <f t="shared" si="1"/>
+        <v>-24034.863354037268</v>
+      </c>
+      <c r="G16">
+        <f t="shared" si="0"/>
+        <v>-16489.034161490683</v>
+      </c>
+      <c r="H16">
+        <f t="shared" si="3"/>
+        <v>267274.84472049691</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8">
+      <c r="A17">
+        <v>2009</v>
+      </c>
+      <c r="B17">
+        <v>-19998</v>
+      </c>
+      <c r="D17">
+        <f>'inflation-output'!B14</f>
+        <v>1.2065217391304348</v>
+      </c>
+      <c r="E17">
+        <f t="shared" si="1"/>
+        <v>-24128.021739130436</v>
+      </c>
+      <c r="G17">
+        <f t="shared" si="0"/>
+        <v>-16489.034161490683</v>
+      </c>
+      <c r="H17">
+        <f t="shared" si="3"/>
+        <v>267274.84472049691</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8">
+      <c r="A18">
+        <v>2010</v>
+      </c>
+      <c r="B18">
+        <v>-19998</v>
+      </c>
+      <c r="D18">
+        <f>'inflation-output'!B15</f>
+        <v>1.1863354037267082</v>
+      </c>
+      <c r="E18">
+        <f t="shared" si="1"/>
+        <v>-23724.335403726709</v>
+      </c>
+      <c r="G18">
+        <f t="shared" si="0"/>
+        <v>-16489.034161490683</v>
+      </c>
+      <c r="H18">
+        <f t="shared" si="3"/>
+        <v>267274.84472049691</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8">
+      <c r="A19">
+        <v>2011</v>
+      </c>
+      <c r="B19">
+        <v>-19998</v>
+      </c>
+      <c r="D19">
+        <f>'inflation-output'!B16</f>
+        <v>1.1506211180124224</v>
+      </c>
+      <c r="E19">
+        <f t="shared" si="1"/>
+        <v>-23010.121118012423</v>
+      </c>
+      <c r="G19">
+        <f t="shared" si="0"/>
+        <v>-16489.034161490683</v>
+      </c>
+      <c r="H19">
+        <f t="shared" si="3"/>
+        <v>267274.84472049691</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8">
+      <c r="A20">
+        <v>2012</v>
+      </c>
+      <c r="B20">
+        <v>-19998</v>
+      </c>
+      <c r="D20">
+        <f>'inflation-output'!B17</f>
+        <v>1.1273291925465838</v>
+      </c>
+      <c r="E20">
+        <f t="shared" si="1"/>
+        <v>-22544.329192546582</v>
+      </c>
+      <c r="G20">
+        <f t="shared" si="0"/>
+        <v>-16489.034161490683</v>
+      </c>
+      <c r="H20">
+        <f t="shared" si="3"/>
+        <v>267274.84472049691</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8">
+      <c r="A21">
+        <v>2013</v>
+      </c>
+      <c r="B21">
+        <v>-19998</v>
+      </c>
+      <c r="D21">
+        <f>'inflation-output'!B18</f>
+        <v>1.110248447204969</v>
+      </c>
+      <c r="E21">
+        <f t="shared" si="1"/>
+        <v>-22202.748447204969</v>
+      </c>
+      <c r="G21">
+        <f t="shared" si="0"/>
+        <v>-16489.034161490683</v>
+      </c>
+      <c r="H21">
+        <f t="shared" si="3"/>
+        <v>267274.84472049691</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8">
+      <c r="A22">
+        <v>2014</v>
+      </c>
+      <c r="B22">
+        <v>-19998</v>
+      </c>
+      <c r="D22">
+        <f>'inflation-output'!B19</f>
+        <v>1.0931677018633541</v>
+      </c>
+      <c r="E22">
+        <f t="shared" si="1"/>
+        <v>-21861.167701863356</v>
+      </c>
+      <c r="G22">
+        <f t="shared" si="0"/>
+        <v>-16489.034161490683</v>
+      </c>
+      <c r="H22">
+        <f t="shared" si="3"/>
+        <v>267274.84472049691</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
+      <c r="A23">
+        <v>2015</v>
+      </c>
+      <c r="B23">
+        <v>-19998</v>
+      </c>
+      <c r="D23">
+        <f>'inflation-output'!B20</f>
+        <v>1.091614906832298</v>
+      </c>
+      <c r="E23">
+        <f t="shared" si="1"/>
+        <v>-21830.114906832296</v>
+      </c>
+      <c r="G23">
+        <f t="shared" si="0"/>
+        <v>-16489.034161490683</v>
+      </c>
+      <c r="H23">
+        <f t="shared" si="3"/>
+        <v>267274.84472049691</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8">
+      <c r="A24">
+        <v>2016</v>
+      </c>
+      <c r="B24">
+        <v>-19998</v>
+      </c>
+      <c r="D24">
+        <f>'inflation-output'!B21</f>
+        <v>1.0776397515527949</v>
+      </c>
+      <c r="E24">
+        <f t="shared" si="1"/>
+        <v>-21550.639751552793</v>
+      </c>
+      <c r="G24">
+        <f t="shared" si="0"/>
+        <v>-16489.034161490683</v>
+      </c>
+      <c r="H24">
+        <f t="shared" si="3"/>
+        <v>267274.84472049691</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8">
+      <c r="A25">
+        <v>2017</v>
+      </c>
+      <c r="B25">
+        <v>-19998</v>
+      </c>
+      <c r="D25">
+        <f>'inflation-output'!B22</f>
+        <v>1.0543478260869565</v>
+      </c>
+      <c r="E25">
+        <f t="shared" si="1"/>
+        <v>-21084.847826086956</v>
+      </c>
+      <c r="G25">
+        <f t="shared" si="0"/>
+        <v>-16489.034161490683</v>
+      </c>
+      <c r="H25">
+        <f t="shared" si="3"/>
+        <v>267274.84472049691</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8">
+      <c r="A26">
+        <v>2018</v>
+      </c>
+      <c r="B26">
+        <v>-19998</v>
+      </c>
+      <c r="D26">
+        <f>'inflation-output'!B23</f>
+        <v>1.0295031055900621</v>
+      </c>
+      <c r="E26">
+        <f t="shared" si="1"/>
+        <v>-20588.003105590062</v>
+      </c>
+      <c r="G26">
+        <f t="shared" si="0"/>
+        <v>-16489.034161490683</v>
+      </c>
+      <c r="H26">
+        <f t="shared" si="3"/>
+        <v>267274.84472049691</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8">
+      <c r="A27">
+        <v>2019</v>
+      </c>
+      <c r="B27">
+        <v>-19998</v>
+      </c>
+      <c r="D27">
+        <f>'inflation-output'!B24</f>
+        <v>1.0124223602484472</v>
+      </c>
+      <c r="E27">
+        <f t="shared" si="1"/>
+        <v>-20246.422360248449</v>
+      </c>
+      <c r="G27">
+        <f t="shared" si="0"/>
+        <v>-16489.034161490683</v>
+      </c>
+      <c r="H27">
+        <f t="shared" si="3"/>
+        <v>267274.84472049691</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8">
+      <c r="A28">
+        <v>2020</v>
+      </c>
+      <c r="B28">
+        <v>-19998</v>
+      </c>
+      <c r="D28">
+        <f>'inflation-output'!B25</f>
+        <v>1</v>
+      </c>
+      <c r="E28">
+        <f t="shared" si="1"/>
+        <v>-19998</v>
+      </c>
+      <c r="G28">
+        <f t="shared" si="0"/>
+        <v>-16489.034161490683</v>
+      </c>
+      <c r="H28">
+        <f t="shared" si="3"/>
+        <v>267274.84472049691</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8">
+      <c r="A29">
+        <v>2021</v>
+      </c>
+      <c r="B29">
+        <v>-19998</v>
+      </c>
+      <c r="D29">
+        <f>'inflation-output'!B26</f>
+        <v>0.95496894409937894</v>
+      </c>
+      <c r="E29">
+        <f t="shared" si="1"/>
+        <v>-19097.468944099379</v>
+      </c>
+      <c r="G29">
+        <f t="shared" si="0"/>
+        <v>-16489.034161490683</v>
+      </c>
+      <c r="H29">
+        <f t="shared" si="3"/>
+        <v>267274.84472049691</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8">
+      <c r="A30">
+        <v>2022</v>
+      </c>
+      <c r="B30">
+        <v>-19998</v>
+      </c>
+      <c r="D30">
+        <f>'inflation-output'!B27</f>
+        <v>0.88354037267080743</v>
+      </c>
+      <c r="E30">
+        <f t="shared" si="1"/>
+        <v>-17669.040372670806</v>
+      </c>
+      <c r="G30">
+        <f t="shared" si="0"/>
+        <v>-16489.034161490683</v>
+      </c>
+      <c r="H30">
+        <f t="shared" si="3"/>
+        <v>267274.84472049691</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8">
+      <c r="A31">
+        <v>2023</v>
+      </c>
+      <c r="B31">
+        <v>-19998</v>
+      </c>
+      <c r="D31">
+        <f>'inflation-output'!B28</f>
+        <v>0.84937888198757772</v>
+      </c>
+      <c r="E31">
+        <f t="shared" si="1"/>
+        <v>-16985.878881987581</v>
+      </c>
+      <c r="G31">
+        <f t="shared" si="0"/>
+        <v>-16489.034161490683</v>
+      </c>
+      <c r="H31">
+        <f t="shared" si="3"/>
+        <v>267274.84472049691</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8">
+      <c r="A32">
+        <v>2024</v>
+      </c>
+      <c r="B32">
+        <v>-19998</v>
+      </c>
+      <c r="D32">
+        <f>'inflation-output'!B29</f>
+        <v>0.82453416149068326</v>
+      </c>
+      <c r="E32">
+        <f t="shared" si="1"/>
+        <v>-16489.034161490683</v>
+      </c>
+      <c r="G32">
+        <f t="shared" si="0"/>
+        <v>-16489.034161490683</v>
+      </c>
+      <c r="H32">
+        <f t="shared" si="3"/>
+        <v>267274.84472049691</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="E5:E32">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F5:F32">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>